<commit_message>
data: Trading Economics xlsx API 증분 갱신 (2026-09-14) [A-248]
</commit_message>
<xml_diff>
--- a/data/raw/Trading Economics/Markets/Commodities/Industrial/2019~2026_Urea_CBOT_USD Per Ton.xlsx
+++ b/data/raw/Trading Economics/Markets/Commodities/Industrial/2019~2026_Urea_CBOT_USD Per Ton.xlsx
@@ -41375,7 +41375,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L175"/>
+  <dimension ref="A1:L176"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <sheetData>
     <row r="1">
@@ -45536,14 +45536,25 @@
       </c>
     </row>
     <row r="175">
-      <c r="A175" t="n">
+      <c r="A175" s="0" t="n">
         <v>9</v>
       </c>
-      <c r="B175" t="n">
+      <c r="B175" s="0" t="n">
         <v>11</v>
       </c>
-      <c r="F175" t="n">
+      <c r="F175" s="0" t="n">
         <v>450.75</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="n">
+        <v>9</v>
+      </c>
+      <c r="B176" t="n">
+        <v>14</v>
+      </c>
+      <c r="F176" t="n">
+        <v>453</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: Trading Economics xlsx API 증분 갱신 (2026-09-15) [A-248]
</commit_message>
<xml_diff>
--- a/data/raw/Trading Economics/Markets/Commodities/Industrial/2019~2026_Urea_CBOT_USD Per Ton.xlsx
+++ b/data/raw/Trading Economics/Markets/Commodities/Industrial/2019~2026_Urea_CBOT_USD Per Ton.xlsx
@@ -41375,7 +41375,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L176"/>
+  <dimension ref="A1:L177"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <sheetData>
     <row r="1">
@@ -45547,14 +45547,25 @@
       </c>
     </row>
     <row r="176">
-      <c r="A176" t="n">
+      <c r="A176" s="0" t="n">
         <v>9</v>
       </c>
-      <c r="B176" t="n">
+      <c r="B176" s="0" t="n">
         <v>14</v>
       </c>
-      <c r="F176" t="n">
+      <c r="F176" s="0" t="n">
         <v>453</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="n">
+        <v>9</v>
+      </c>
+      <c r="B177" t="n">
+        <v>15</v>
+      </c>
+      <c r="F177" t="n">
+        <v>459.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: Trading Economics xlsx API 증분 갱신 (2026-09-16) [A-248]
</commit_message>
<xml_diff>
--- a/data/raw/Trading Economics/Markets/Commodities/Industrial/2019~2026_Urea_CBOT_USD Per Ton.xlsx
+++ b/data/raw/Trading Economics/Markets/Commodities/Industrial/2019~2026_Urea_CBOT_USD Per Ton.xlsx
@@ -41375,7 +41375,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L177"/>
+  <dimension ref="A1:L178"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <sheetData>
     <row r="1">
@@ -45558,14 +45558,25 @@
       </c>
     </row>
     <row r="177">
-      <c r="A177" t="n">
+      <c r="A177" s="0" t="n">
         <v>9</v>
       </c>
-      <c r="B177" t="n">
+      <c r="B177" s="0" t="n">
         <v>15</v>
       </c>
-      <c r="F177" t="n">
+      <c r="F177" s="0" t="n">
         <v>459.5</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="n">
+        <v>9</v>
+      </c>
+      <c r="B178" t="n">
+        <v>16</v>
+      </c>
+      <c r="F178" t="n">
+        <v>460</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: Trading Economics xlsx API 증분 갱신 (2026-09-17) [A-248]
</commit_message>
<xml_diff>
--- a/data/raw/Trading Economics/Markets/Commodities/Industrial/2019~2026_Urea_CBOT_USD Per Ton.xlsx
+++ b/data/raw/Trading Economics/Markets/Commodities/Industrial/2019~2026_Urea_CBOT_USD Per Ton.xlsx
@@ -41375,7 +41375,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L178"/>
+  <dimension ref="A1:L179"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <sheetData>
     <row r="1">
@@ -45569,14 +45569,25 @@
       </c>
     </row>
     <row r="178">
-      <c r="A178" t="n">
+      <c r="A178" s="0" t="n">
         <v>9</v>
       </c>
-      <c r="B178" t="n">
+      <c r="B178" s="0" t="n">
         <v>16</v>
       </c>
-      <c r="F178" t="n">
+      <c r="F178" s="0" t="n">
         <v>460</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="n">
+        <v>9</v>
+      </c>
+      <c r="B179" t="n">
+        <v>17</v>
+      </c>
+      <c r="F179" t="n">
+        <v>460.25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: Trading Economics xlsx API 증분 갱신 (2026-09-18) [A-248]
</commit_message>
<xml_diff>
--- a/data/raw/Trading Economics/Markets/Commodities/Industrial/2019~2026_Urea_CBOT_USD Per Ton.xlsx
+++ b/data/raw/Trading Economics/Markets/Commodities/Industrial/2019~2026_Urea_CBOT_USD Per Ton.xlsx
@@ -41375,7 +41375,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L179"/>
+  <dimension ref="A1:L180"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <sheetData>
     <row r="1">
@@ -45580,14 +45580,25 @@
       </c>
     </row>
     <row r="179">
-      <c r="A179" t="n">
+      <c r="A179" s="0" t="n">
         <v>9</v>
       </c>
-      <c r="B179" t="n">
+      <c r="B179" s="0" t="n">
         <v>17</v>
       </c>
-      <c r="F179" t="n">
+      <c r="F179" s="0" t="n">
         <v>460.25</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="n">
+        <v>9</v>
+      </c>
+      <c r="B180" t="n">
+        <v>18</v>
+      </c>
+      <c r="F180" t="n">
+        <v>459.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: Trading Economics xlsx API 증분 갱신 (2026-09-22) [A-248]
</commit_message>
<xml_diff>
--- a/data/raw/Trading Economics/Markets/Commodities/Industrial/2019~2026_Urea_CBOT_USD Per Ton.xlsx
+++ b/data/raw/Trading Economics/Markets/Commodities/Industrial/2019~2026_Urea_CBOT_USD Per Ton.xlsx
@@ -41375,7 +41375,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L180"/>
+  <dimension ref="A1:L181"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <sheetData>
     <row r="1">
@@ -45591,14 +45591,25 @@
       </c>
     </row>
     <row r="180">
-      <c r="A180" t="n">
+      <c r="A180" s="0" t="n">
         <v>9</v>
       </c>
-      <c r="B180" t="n">
+      <c r="B180" s="0" t="n">
         <v>18</v>
       </c>
-      <c r="F180" t="n">
+      <c r="F180" s="0" t="n">
         <v>459.5</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="n">
+        <v>9</v>
+      </c>
+      <c r="B181" t="n">
+        <v>21</v>
+      </c>
+      <c r="F181" t="n">
+        <v>460</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: Trading Economics xlsx API 증분 갱신 (2026-09-23) [A-248]
</commit_message>
<xml_diff>
--- a/data/raw/Trading Economics/Markets/Commodities/Industrial/2019~2026_Urea_CBOT_USD Per Ton.xlsx
+++ b/data/raw/Trading Economics/Markets/Commodities/Industrial/2019~2026_Urea_CBOT_USD Per Ton.xlsx
@@ -41375,7 +41375,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L181"/>
+  <dimension ref="A1:L182"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <sheetData>
     <row r="1">
@@ -45602,14 +45602,25 @@
       </c>
     </row>
     <row r="181">
-      <c r="A181" t="n">
+      <c r="A181" s="0" t="n">
         <v>9</v>
       </c>
-      <c r="B181" t="n">
+      <c r="B181" s="0" t="n">
         <v>21</v>
       </c>
-      <c r="F181" t="n">
+      <c r="F181" s="0" t="n">
         <v>460</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="n">
+        <v>9</v>
+      </c>
+      <c r="B182" t="n">
+        <v>23</v>
+      </c>
+      <c r="F182" t="n">
+        <v>458</v>
       </c>
     </row>
   </sheetData>

</xml_diff>